<commit_message>
JS function and structure
</commit_message>
<xml_diff>
--- a/LB_Program_Statements.xlsx
+++ b/LB_Program_Statements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHREYA\Desktop\LB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FA8B4F5-12F1-4F30-803C-B3D287941A7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{114B9998-3E40-4402-9013-4DFFA78BAE16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11295" xr2:uid="{529304FC-C76E-4A78-91F7-2381E30A6342}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1674" uniqueCount="877">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1689" uniqueCount="886">
   <si>
     <t>Jay Ganesh print in c</t>
   </si>
@@ -3550,6 +3550,33 @@
   </si>
   <si>
     <t>for loop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">perfect number function usung for loop </t>
+  </si>
+  <si>
+    <t xml:space="preserve">addtion of factors is equal to number itself </t>
+  </si>
+  <si>
+    <t>while loop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">digits summation function </t>
+  </si>
+  <si>
+    <t>Array let Arr = [ 12,23]</t>
+  </si>
+  <si>
+    <t>jS</t>
+  </si>
+  <si>
+    <t>typeof inbuild function</t>
+  </si>
+  <si>
+    <t>String traversal</t>
+  </si>
+  <si>
+    <t>count small characters are</t>
   </si>
 </sst>
 </file>
@@ -4000,7 +4027,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099BD82-CF9E-4D41-BD71-1A037607BD64}">
-  <dimension ref="A1:C1033"/>
+  <dimension ref="A1:C1046"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="106.140625" bestFit="1" customWidth="1"/>
@@ -10638,7 +10665,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="1028" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1028" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1028" t="s">
         <v>872</v>
       </c>
@@ -10646,7 +10673,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="1029" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1029" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1029" t="s">
         <v>873</v>
       </c>
@@ -10654,7 +10681,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="1030" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1030" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1030" t="s">
         <v>875</v>
       </c>
@@ -10662,12 +10689,71 @@
         <v>874</v>
       </c>
     </row>
-    <row r="1033" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1033" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1033" t="s">
         <v>876</v>
       </c>
       <c r="B1033" t="s">
         <v>869</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1035" t="s">
+        <v>877</v>
+      </c>
+      <c r="B1035" t="s">
+        <v>874</v>
+      </c>
+      <c r="C1035" t="s">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="1036" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1036" t="s">
+        <v>879</v>
+      </c>
+      <c r="B1036" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="1037" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1037" t="s">
+        <v>880</v>
+      </c>
+      <c r="B1037" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="1039" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1039" t="s">
+        <v>881</v>
+      </c>
+      <c r="B1039" t="s">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="1040" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1040" t="s">
+        <v>883</v>
+      </c>
+      <c r="B1040" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="1045" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1045" t="s">
+        <v>884</v>
+      </c>
+      <c r="B1045" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1046" t="s">
+        <v>885</v>
+      </c>
+      <c r="B1046" t="s">
+        <v>874</v>
       </c>
     </row>
   </sheetData>

</xml_diff>